<commit_message>
Page 4: review and map
Task workspace step 2 for SFS tasks: entity tabs, translation rates panel (cross rates
from the USD master, historical rate from the entity master), accounts to map with FSLI
suggestions and server-side validation, TB with mapping (filters, reasoned changes),
FSLI and intercompany summaries, and continue to comparatives. Configuration shows each
entity's chart of accounts with mapping source.

Engine: crossRate, periodUsdRate, accountsToMap, suggestFsli, validateMapping,
fsliTotals, intercompanySummary (unit-tested). Sample data revised so the expected
Aug-2026 results (IN totals, profit, IC balances, rates; UK profit) hold exactly and are
asserted in API tests.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/Chart_of_Accounts_IN_sample.xlsx
+++ b/samples/Chart_of_Accounts_IN_sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D42"/>
   <cols>
     <col min="1" max="1" width="52.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -575,10 +575,10 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Advance to Suppliers</v>
+        <v>Due from Aistra Labs AI Software LLC (UAE)</v>
       </c>
       <c r="B13" t="str">
-        <v>1455</v>
+        <v>1452</v>
       </c>
       <c r="C13" t="str">
         <v>Other Current Asset</v>
@@ -589,13 +589,13 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Computers and Equipment</v>
+        <v>Due from Unconstrained INC</v>
       </c>
       <c r="B14" t="str">
-        <v>1500</v>
+        <v>1453</v>
       </c>
       <c r="C14" t="str">
-        <v>Fixed Asset</v>
+        <v>Other Current Asset</v>
       </c>
       <c r="D14" t="str">
         <v/>
@@ -603,13 +603,13 @@
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Accumulated Depreciation - Computers and Equipment</v>
+        <v>Advance to Suppliers</v>
       </c>
       <c r="B15" t="str">
-        <v>1510</v>
+        <v>1455</v>
       </c>
       <c r="C15" t="str">
-        <v>Fixed Asset</v>
+        <v>Other Current Asset</v>
       </c>
       <c r="D15" t="str">
         <v/>
@@ -617,13 +617,13 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Deferred Tax Asset</v>
+        <v>Computers and Equipment</v>
       </c>
       <c r="B16" t="str">
-        <v>1600</v>
+        <v>1500</v>
       </c>
       <c r="C16" t="str">
-        <v>Other Asset</v>
+        <v>Fixed Asset</v>
       </c>
       <c r="D16" t="str">
         <v/>
@@ -631,13 +631,13 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Accounts Payable</v>
+        <v>Accumulated Depreciation - Computers and Equipment</v>
       </c>
       <c r="B17" t="str">
-        <v>2001</v>
+        <v>1510</v>
       </c>
       <c r="C17" t="str">
-        <v>Accounts Payable</v>
+        <v>Fixed Asset</v>
       </c>
       <c r="D17" t="str">
         <v/>
@@ -645,13 +645,13 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Accrued Expenses</v>
+        <v>Deferred Tax Asset</v>
       </c>
       <c r="B18" t="str">
-        <v>2100</v>
+        <v>1600</v>
       </c>
       <c r="C18" t="str">
-        <v>Other Current Liability</v>
+        <v>Other Asset</v>
       </c>
       <c r="D18" t="str">
         <v/>
@@ -659,13 +659,13 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Income Tax Payable</v>
+        <v>Accounts Payable</v>
       </c>
       <c r="B19" t="str">
-        <v>2150</v>
+        <v>2001</v>
       </c>
       <c r="C19" t="str">
-        <v>Other Current Liability</v>
+        <v>Accounts Payable</v>
       </c>
       <c r="D19" t="str">
         <v/>
@@ -673,10 +673,10 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Provision for Leave Encashment</v>
+        <v>Accrued Expenses</v>
       </c>
       <c r="B20" t="str">
-        <v>2200</v>
+        <v>2100</v>
       </c>
       <c r="C20" t="str">
         <v>Other Current Liability</v>
@@ -687,13 +687,13 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Equity Share Capital</v>
+        <v>Income Tax Payable</v>
       </c>
       <c r="B21" t="str">
-        <v>3001</v>
+        <v>2150</v>
       </c>
       <c r="C21" t="str">
-        <v>Equity</v>
+        <v>Other Current Liability</v>
       </c>
       <c r="D21" t="str">
         <v/>
@@ -701,13 +701,13 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Securities Premium</v>
+        <v>Provision for Leave Encashment</v>
       </c>
       <c r="B22" t="str">
-        <v>3100</v>
+        <v>2200</v>
       </c>
       <c r="C22" t="str">
-        <v>Equity</v>
+        <v>Other Current Liability</v>
       </c>
       <c r="D22" t="str">
         <v/>
@@ -715,10 +715,10 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Retained Earnings</v>
+        <v>Equity Share Capital</v>
       </c>
       <c r="B23" t="str">
-        <v>3200</v>
+        <v>3001</v>
       </c>
       <c r="C23" t="str">
         <v>Equity</v>
@@ -729,13 +729,13 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Consulting Revenue</v>
+        <v>Securities Premium</v>
       </c>
       <c r="B24" t="str">
-        <v>4001</v>
+        <v>3100</v>
       </c>
       <c r="C24" t="str">
-        <v>Income</v>
+        <v>Equity</v>
       </c>
       <c r="D24" t="str">
         <v/>
@@ -743,13 +743,13 @@
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>IC Revenue - US</v>
+        <v>Retained Earnings</v>
       </c>
       <c r="B25" t="str">
-        <v>4100</v>
+        <v>3200</v>
       </c>
       <c r="C25" t="str">
-        <v>Income</v>
+        <v>Equity</v>
       </c>
       <c r="D25" t="str">
         <v/>
@@ -757,10 +757,10 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>IC Revenue - UK</v>
+        <v>Consulting Revenue</v>
       </c>
       <c r="B26" t="str">
-        <v>4101</v>
+        <v>4001</v>
       </c>
       <c r="C26" t="str">
         <v>Income</v>
@@ -771,13 +771,13 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>Interest Income</v>
+        <v>IC Revenue - US</v>
       </c>
       <c r="B27" t="str">
-        <v>4500</v>
+        <v>4100</v>
       </c>
       <c r="C27" t="str">
-        <v>Other Income</v>
+        <v>Income</v>
       </c>
       <c r="D27" t="str">
         <v/>
@@ -785,13 +785,13 @@
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>Cost of Services</v>
+        <v>IC Revenue - UK</v>
       </c>
       <c r="B28" t="str">
-        <v>5001</v>
+        <v>4101</v>
       </c>
       <c r="C28" t="str">
-        <v>Cost Of Goods Sold</v>
+        <v>Income</v>
       </c>
       <c r="D28" t="str">
         <v/>
@@ -799,13 +799,13 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>Salaries and Wages</v>
+        <v>IC Revenue - UAE</v>
       </c>
       <c r="B29" t="str">
-        <v>6001</v>
+        <v>4102</v>
       </c>
       <c r="C29" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D29" t="str">
         <v/>
@@ -813,13 +813,13 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Travel and Conveyance</v>
+        <v>IC Revenue - Unconstrained</v>
       </c>
       <c r="B30" t="str">
-        <v>6100</v>
+        <v>4103</v>
       </c>
       <c r="C30" t="str">
-        <v>Expense</v>
+        <v>Income</v>
       </c>
       <c r="D30" t="str">
         <v/>
@@ -827,13 +827,13 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>Staff Welfare Expenses</v>
+        <v>Interest Income</v>
       </c>
       <c r="B31" t="str">
-        <v>6120</v>
+        <v>4500</v>
       </c>
       <c r="C31" t="str">
-        <v>Expense</v>
+        <v>Other Income</v>
       </c>
       <c r="D31" t="str">
         <v/>
@@ -841,13 +841,13 @@
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>Professional Fees</v>
+        <v>Cost of Services</v>
       </c>
       <c r="B32" t="str">
-        <v>6200</v>
+        <v>5001</v>
       </c>
       <c r="C32" t="str">
-        <v>Expense</v>
+        <v>Cost Of Goods Sold</v>
       </c>
       <c r="D32" t="str">
         <v/>
@@ -855,10 +855,10 @@
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>Software Subscriptions</v>
+        <v>Salaries and Wages</v>
       </c>
       <c r="B33" t="str">
-        <v>6300</v>
+        <v>6001</v>
       </c>
       <c r="C33" t="str">
         <v>Expense</v>
@@ -869,10 +869,10 @@
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>Rent</v>
+        <v>Travel and Conveyance</v>
       </c>
       <c r="B34" t="str">
-        <v>6400</v>
+        <v>6100</v>
       </c>
       <c r="C34" t="str">
         <v>Expense</v>
@@ -883,10 +883,10 @@
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>Depreciation</v>
+        <v>Staff Welfare Expenses</v>
       </c>
       <c r="B35" t="str">
-        <v>6500</v>
+        <v>6120</v>
       </c>
       <c r="C35" t="str">
         <v>Expense</v>
@@ -897,10 +897,10 @@
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>Income Tax Expense</v>
+        <v>Professional Fees</v>
       </c>
       <c r="B36" t="str">
-        <v>6900</v>
+        <v>6200</v>
       </c>
       <c r="C36" t="str">
         <v>Expense</v>
@@ -911,10 +911,10 @@
     </row>
     <row r="37">
       <c r="A37" t="str">
-        <v>Office Supplies</v>
+        <v>Software Subscriptions</v>
       </c>
       <c r="B37" t="str">
-        <v>6150</v>
+        <v>6300</v>
       </c>
       <c r="C37" t="str">
         <v>Expense</v>
@@ -925,21 +925,77 @@
     </row>
     <row r="38">
       <c r="A38" t="str">
+        <v>Rent</v>
+      </c>
+      <c r="B38" t="str">
+        <v>6400</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D38" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Depreciation</v>
+      </c>
+      <c r="B39" t="str">
+        <v>6500</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D39" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Income Tax Expense</v>
+      </c>
+      <c r="B40" t="str">
+        <v>6900</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D40" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Office Supplies</v>
+      </c>
+      <c r="B41" t="str">
+        <v>6150</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Expense</v>
+      </c>
+      <c r="D41" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
         <v>Fixed Deposit - HDFC</v>
       </c>
-      <c r="B38" t="str">
+      <c r="B42" t="str">
         <v>1060</v>
       </c>
-      <c r="C38" t="str">
+      <c r="C42" t="str">
         <v>Bank</v>
       </c>
-      <c r="D38" t="str">
+      <c r="D42" t="str">
         <v>HDFC Bank Current Account</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D38"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D42"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>